<commit_message>
Day 3 Functions Lists and Employee Salary Analysis completed
</commit_message>
<xml_diff>
--- a/excel/employee_data.xlsx
+++ b/excel/employee_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data_analyst_journey2026\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CFA32DB-D16A-4366-9FD4-F28271B886C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8F43C1-906C-44B0-A1EA-E68DA56A4265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E5E5196-FBF7-49AE-88D8-ECA945F973E1}"/>
   </bookViews>
@@ -182,7 +182,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -221,7 +221,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>